<commit_message>
Add app manual review scoring
</commit_message>
<xml_diff>
--- a/experiments/Experimental_results.xlsx
+++ b/experiments/Experimental_results.xlsx
@@ -2,7 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Model_Selection" sheetId="1" r:id="Rc63692fb28904d19"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Model_Selection" sheetId="1" r:id="R45888a6049d44b4b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Streamlit_App_Tests" sheetId="2" r:id="Rf3b9fcf0835e4831"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Manual_Review_Scoring" sheetId="3" r:id="R4b776c825f444c15"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -221,7 +223,7 @@
       </x:c>
     </x:row>
     <x:row r="2">
-      <x:c r="A2" t="str">
+      <x:c r="A2" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="B2" t="str">
@@ -233,16 +235,16 @@
       <x:c r="D2" t="str">
         <x:v>CPU</x:v>
       </x:c>
-      <x:c r="E2" t="str">
+      <x:c r="E2" t="n">
         <x:v>455</x:v>
       </x:c>
-      <x:c r="F2" t="str">
+      <x:c r="F2" t="n">
         <x:v>0.7033</x:v>
       </x:c>
-      <x:c r="G2" t="str">
+      <x:c r="G2" t="n">
         <x:v>38.6122</x:v>
       </x:c>
-      <x:c r="H2" t="str">
+      <x:c r="H2" t="n">
         <x:v>27.8509</x:v>
       </x:c>
       <x:c r="I2" t="str">
@@ -250,7 +252,7 @@
       </x:c>
     </x:row>
     <x:row r="3">
-      <x:c r="A3" t="str">
+      <x:c r="A3" t="n">
         <x:v>2</x:v>
       </x:c>
       <x:c r="B3" t="str">
@@ -262,16 +264,16 @@
       <x:c r="D3" t="str">
         <x:v>GPU</x:v>
       </x:c>
-      <x:c r="E3" t="str">
+      <x:c r="E3" t="n">
         <x:v>455</x:v>
       </x:c>
-      <x:c r="F3" t="str">
+      <x:c r="F3" t="n">
         <x:v>0.7033</x:v>
       </x:c>
-      <x:c r="G3" t="str">
+      <x:c r="G3" t="n">
         <x:v>4.8555</x:v>
       </x:c>
-      <x:c r="H3" t="str">
+      <x:c r="H3" t="n">
         <x:v>3.9927</x:v>
       </x:c>
       <x:c r="I3" t="str">
@@ -279,7 +281,7 @@
       </x:c>
     </x:row>
     <x:row r="4">
-      <x:c r="A4" t="str">
+      <x:c r="A4" t="n">
         <x:v>3</x:v>
       </x:c>
       <x:c r="B4" t="str">
@@ -291,16 +293,16 @@
       <x:c r="D4" t="str">
         <x:v>CPU</x:v>
       </x:c>
-      <x:c r="E4" t="str">
+      <x:c r="E4" t="n">
         <x:v>455</x:v>
       </x:c>
-      <x:c r="F4" t="str">
+      <x:c r="F4" t="n">
         <x:v>0.7604</x:v>
       </x:c>
-      <x:c r="G4" t="str">
+      <x:c r="G4" t="n">
         <x:v>30.7984</x:v>
       </x:c>
-      <x:c r="H4" t="str">
+      <x:c r="H4" t="n">
         <x:v>25.9997</x:v>
       </x:c>
       <x:c r="I4" t="str">
@@ -308,7 +310,7 @@
       </x:c>
     </x:row>
     <x:row r="5">
-      <x:c r="A5" t="str">
+      <x:c r="A5" t="n">
         <x:v>4</x:v>
       </x:c>
       <x:c r="B5" t="str">
@@ -320,16 +322,16 @@
       <x:c r="D5" t="str">
         <x:v>GPU</x:v>
       </x:c>
-      <x:c r="E5" t="str">
+      <x:c r="E5" t="n">
         <x:v>455</x:v>
       </x:c>
-      <x:c r="F5" t="str">
+      <x:c r="F5" t="n">
         <x:v>0.7604</x:v>
       </x:c>
-      <x:c r="G5" t="str">
+      <x:c r="G5" t="n">
         <x:v>3.2396</x:v>
       </x:c>
-      <x:c r="H5" t="str">
+      <x:c r="H5" t="n">
         <x:v>2.2477</x:v>
       </x:c>
       <x:c r="I5" t="str">
@@ -337,7 +339,7 @@
       </x:c>
     </x:row>
     <x:row r="6">
-      <x:c r="A6" t="str">
+      <x:c r="A6" t="n">
         <x:v>5</x:v>
       </x:c>
       <x:c r="B6" t="str">
@@ -349,24 +351,24 @@
       <x:c r="D6" t="str">
         <x:v>CPU</x:v>
       </x:c>
-      <x:c r="E6" t="str">
+      <x:c r="E6" t="n">
         <x:v>455</x:v>
       </x:c>
-      <x:c r="F6" t="str">
+      <x:c r="F6" t="n">
         <x:v>0.7363</x:v>
       </x:c>
-      <x:c r="G6" t="str">
+      <x:c r="G6" t="n">
         <x:v>57.5298</x:v>
       </x:c>
-      <x:c r="H6" t="str">
-        <x:v>50.5400</x:v>
+      <x:c r="H6" t="n">
+        <x:v>50.54</x:v>
       </x:c>
       <x:c r="I6" t="str">
         <x:v>Sentiment pipeline as supporting signal</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
-      <x:c r="A7" t="str">
+      <x:c r="A7" t="n">
         <x:v>6</x:v>
       </x:c>
       <x:c r="B7" t="str">
@@ -378,20 +380,342 @@
       <x:c r="D7" t="str">
         <x:v>GPU</x:v>
       </x:c>
-      <x:c r="E7" t="str">
+      <x:c r="E7" t="n">
         <x:v>455</x:v>
       </x:c>
-      <x:c r="F7" t="str">
+      <x:c r="F7" t="n">
         <x:v>0.7363</x:v>
       </x:c>
-      <x:c r="G7" t="str">
-        <x:v>6.1080</x:v>
-      </x:c>
-      <x:c r="H7" t="str">
+      <x:c r="G7" t="n">
+        <x:v>6.108</x:v>
+      </x:c>
+      <x:c r="H7" t="n">
         <x:v>4.2489</x:v>
       </x:c>
       <x:c r="I7" t="str">
         <x:v>Sentiment pipeline on GPU</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:sheetData>
+    <x:row r="1">
+      <x:c r="A1" t="str">
+        <x:v>video</x:v>
+      </x:c>
+      <x:c r="B1" t="str">
+        <x:v>num_comments</x:v>
+      </x:c>
+      <x:c r="C1" t="str">
+        <x:v>app_main_emotion</x:v>
+      </x:c>
+      <x:c r="D1" t="str">
+        <x:v>manual_main_emotion</x:v>
+      </x:c>
+      <x:c r="E1" t="str">
+        <x:v>correct</x:v>
+      </x:c>
+      <x:c r="F1" t="str">
+        <x:v>negative_emotion_ratio</x:v>
+      </x:c>
+      <x:c r="G1" t="str">
+        <x:v>anger_pct</x:v>
+      </x:c>
+      <x:c r="H1" t="str">
+        <x:v>disgust_pct</x:v>
+      </x:c>
+      <x:c r="I1" t="str">
+        <x:v>fear_pct</x:v>
+      </x:c>
+      <x:c r="J1" t="str">
+        <x:v>joy_pct</x:v>
+      </x:c>
+      <x:c r="K1" t="str">
+        <x:v>neutral_pct</x:v>
+      </x:c>
+      <x:c r="L1" t="str">
+        <x:v>sadness_pct</x:v>
+      </x:c>
+      <x:c r="M1" t="str">
+        <x:v>surprise_pct</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2">
+      <x:c r="A2" t="str">
+        <x:v>https://www.youtube.com/watch?v=d2dgJGkw5p0</x:v>
+      </x:c>
+      <x:c r="B2" t="n">
+        <x:v>50</x:v>
+      </x:c>
+      <x:c r="C2" t="str">
+        <x:v>neutral</x:v>
+      </x:c>
+      <x:c r="D2" t="str">
+        <x:v>neutral</x:v>
+      </x:c>
+      <x:c r="E2" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="F2" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="G2" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="H2" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="I2" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J2" t="n">
+        <x:v>14</x:v>
+      </x:c>
+      <x:c r="K2" t="n">
+        <x:v>70</x:v>
+      </x:c>
+      <x:c r="L2" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="M2" t="n">
+        <x:v>6</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3">
+      <x:c r="A3" t="str">
+        <x:v>https://www.youtube.com/watch?v=M8To7iorkxQ</x:v>
+      </x:c>
+      <x:c r="B3" t="n">
+        <x:v>50</x:v>
+      </x:c>
+      <x:c r="C3" t="str">
+        <x:v>neutral</x:v>
+      </x:c>
+      <x:c r="D3" t="str">
+        <x:v>joy</x:v>
+      </x:c>
+      <x:c r="E3" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="F3" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="G3" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="H3" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I3" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J3" t="n">
+        <x:v>24</x:v>
+      </x:c>
+      <x:c r="K3" t="n">
+        <x:v>64</x:v>
+      </x:c>
+      <x:c r="L3" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="M3" t="n">
+        <x:v>8</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4">
+      <x:c r="A4" t="str">
+        <x:v>https://www.youtube.com/watch?v=-_-eIVAX1yQ</x:v>
+      </x:c>
+      <x:c r="B4" t="n">
+        <x:v>50</x:v>
+      </x:c>
+      <x:c r="C4" t="str">
+        <x:v>neutral</x:v>
+      </x:c>
+      <x:c r="D4" t="str">
+        <x:v>anger</x:v>
+      </x:c>
+      <x:c r="E4" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="F4" t="n">
+        <x:v>28</x:v>
+      </x:c>
+      <x:c r="G4" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="H4" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="I4" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="J4" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="K4" t="n">
+        <x:v>62</x:v>
+      </x:c>
+      <x:c r="L4" t="n">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="M4" t="n">
+        <x:v>8</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:sheetData>
+    <x:row r="1">
+      <x:c r="A1" t="str">
+        <x:v>video</x:v>
+      </x:c>
+      <x:c r="B1" t="str">
+        <x:v>num_comments</x:v>
+      </x:c>
+      <x:c r="C1" t="str">
+        <x:v>manual_7_emotion</x:v>
+      </x:c>
+      <x:c r="D1" t="str">
+        <x:v>manual_7_score</x:v>
+      </x:c>
+      <x:c r="E1" t="str">
+        <x:v>app_7_emotion</x:v>
+      </x:c>
+      <x:c r="F1" t="str">
+        <x:v>emotion_correct</x:v>
+      </x:c>
+      <x:c r="G1" t="str">
+        <x:v>manual_3_sentiment</x:v>
+      </x:c>
+      <x:c r="H1" t="str">
+        <x:v>manual_3_score</x:v>
+      </x:c>
+      <x:c r="I1" t="str">
+        <x:v>app_3_sentiment</x:v>
+      </x:c>
+      <x:c r="J1" t="str">
+        <x:v>sentiment_correct</x:v>
+      </x:c>
+      <x:c r="K1" t="str">
+        <x:v>rationale</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2">
+      <x:c r="A2" t="str">
+        <x:v>https://www.youtube.com/watch?v=d2dgJGkw5p0</x:v>
+      </x:c>
+      <x:c r="B2" t="n">
+        <x:v>50</x:v>
+      </x:c>
+      <x:c r="C2" t="str">
+        <x:v>neutral</x:v>
+      </x:c>
+      <x:c r="D2" t="n">
+        <x:v>68</x:v>
+      </x:c>
+      <x:c r="E2" t="str">
+        <x:v>neutral</x:v>
+      </x:c>
+      <x:c r="F2" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="G2" t="str">
+        <x:v>neutral</x:v>
+      </x:c>
+      <x:c r="H2" t="n">
+        <x:v>62</x:v>
+      </x:c>
+      <x:c r="I2" t="str">
+        <x:v>neutral</x:v>
+      </x:c>
+      <x:c r="J2" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="K2" t="str">
+        <x:v>Mostly informational and geopolitical discussion; some sarcasm and criticism are present, but no single strong emotion dominates.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3">
+      <x:c r="A3" t="str">
+        <x:v>https://www.youtube.com/watch?v=M8To7iorkxQ</x:v>
+      </x:c>
+      <x:c r="B3" t="n">
+        <x:v>50</x:v>
+      </x:c>
+      <x:c r="C3" t="str">
+        <x:v>joy</x:v>
+      </x:c>
+      <x:c r="D3" t="n">
+        <x:v>88</x:v>
+      </x:c>
+      <x:c r="E3" t="str">
+        <x:v>neutral</x:v>
+      </x:c>
+      <x:c r="F3" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="G3" t="str">
+        <x:v>positive</x:v>
+      </x:c>
+      <x:c r="H3" t="n">
+        <x:v>92</x:v>
+      </x:c>
+      <x:c r="I3" t="str">
+        <x:v>positive</x:v>
+      </x:c>
+      <x:c r="J3" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="K3" t="str">
+        <x:v>Many comments praise the video or movie, use hearts, and contain positive wording such as amazing, enjoying, and favorite.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4">
+      <x:c r="A4" t="str">
+        <x:v>https://www.youtube.com/watch?v=-_-eIVAX1yQ</x:v>
+      </x:c>
+      <x:c r="B4" t="n">
+        <x:v>50</x:v>
+      </x:c>
+      <x:c r="C4" t="str">
+        <x:v>anger</x:v>
+      </x:c>
+      <x:c r="D4" t="n">
+        <x:v>72</x:v>
+      </x:c>
+      <x:c r="E4" t="str">
+        <x:v>neutral</x:v>
+      </x:c>
+      <x:c r="F4" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="G4" t="str">
+        <x:v>negative</x:v>
+      </x:c>
+      <x:c r="H4" t="n">
+        <x:v>85</x:v>
+      </x:c>
+      <x:c r="I4" t="str">
+        <x:v>negative</x:v>
+      </x:c>
+      <x:c r="J4" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="K4" t="str">
+        <x:v>Comments include blame, insults, political hostility, and violent sarcasm; negative anger dominates despite some dark humor.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
Add all 5 models to report, experiments, and testing notebook
- Update Project_report_skeleton.md with SamLowe and RoBERTa-large rows
- Add app_model_comparison_5models.csv with full 5-model results
- Update Experimental_results.xlsx with App_5Model_Comparison sheet
- Update testing_experiments.ipynb cell 26 with all 5 models
- Regenerate Project_report.pdf (8 pages)

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/experiments/Experimental_results.xlsx
+++ b/experiments/Experimental_results.xlsx
@@ -9,8 +9,9 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Model_Selection" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Streamlit_App_Performance" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="App_Runtime" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Manual_Comment_Labels" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="App_5Model_Comparison" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="App_Runtime" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Manual_Comment_Labels" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -446,14 +447,14 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
-    <col width="40" customWidth="1" min="2" max="2"/>
+    <col width="45" customWidth="1" min="2" max="2"/>
     <col width="30" customWidth="1" min="3" max="3"/>
     <col width="8" customWidth="1" min="4" max="4"/>
     <col width="18" customWidth="1" min="5" max="5"/>
     <col width="10" customWidth="1" min="6" max="6"/>
     <col width="36" customWidth="1" min="7" max="7"/>
     <col width="39" customWidth="1" min="8" max="8"/>
-    <col width="40" customWidth="1" min="9" max="9"/>
+    <col width="45" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -813,10 +814,10 @@
   <dimension ref="A1:I17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="40" customWidth="1" min="1" max="1"/>
+    <col width="45" customWidth="1" min="1" max="1"/>
     <col width="17" customWidth="1" min="2" max="2"/>
     <col width="32" customWidth="1" min="3" max="3"/>
-    <col width="40" customWidth="1" min="4" max="4"/>
+    <col width="45" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
     <col width="18" customWidth="1" min="6" max="6"/>
     <col width="10" customWidth="1" min="7" max="7"/>
@@ -1522,239 +1523,842 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G7"/>
+  <dimension ref="A1:I22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="40" customWidth="1" min="1" max="1"/>
+    <col width="45" customWidth="1" min="1" max="1"/>
     <col width="37" customWidth="1" min="2" max="2"/>
-    <col width="8" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="36" customWidth="1" min="5" max="5"/>
-    <col width="39" customWidth="1" min="6" max="6"/>
-    <col width="36" customWidth="1" min="7" max="7"/>
+    <col width="45" customWidth="1" min="3" max="3"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="9" customWidth="1" min="5" max="5"/>
+    <col width="7" customWidth="1" min="6" max="6"/>
+    <col width="20" customWidth="1" min="7" max="7"/>
+    <col width="8" customWidth="1" min="8" max="8"/>
+    <col width="9" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>model_name</t>
+          <t>video</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>dataset</t>
+          <t>model</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>device</t>
+          <t>repo</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>num_comments</t>
+          <t>task</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>runtime_with_model_loading_seconds</t>
+          <t>matched</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>runtime_without_model_loading_seconds</t>
+          <t>total</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>notes</t>
+          <t>accuracy</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>load_s</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>infer_s</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
+          <t>https://www.youtube.com/watch?v=d2dgJGkw5p0</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Pre-tuning baseline</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
           <t>j-hartmann/emotion-english-distilroberta-base</t>
         </is>
       </c>
-      <c r="B2" s="2" t="inlineStr">
-        <is>
-          <t>150 reviewed Streamlit app comments</t>
-        </is>
-      </c>
-      <c r="C2" s="2" t="inlineStr">
-        <is>
-          <t>CPU</t>
-        </is>
-      </c>
-      <c r="D2" s="2" t="n">
-        <v>150</v>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>7-emotion</t>
+        </is>
       </c>
       <c r="E2" s="2" t="n">
-        <v>7.2815</v>
+        <v>29</v>
       </c>
       <c r="F2" s="2" t="n">
-        <v>1.5164</v>
-      </c>
-      <c r="G2" s="2" t="inlineStr">
-        <is>
-          <t>pre-tuning public baseline</t>
-        </is>
+        <v>50</v>
+      </c>
+      <c r="G2" s="2" t="n">
+        <v>0.58</v>
+      </c>
+      <c r="H2" s="2" t="n">
+        <v>1.48</v>
+      </c>
+      <c r="I2" s="2" t="n">
+        <v>1.52</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>chase1zhang/youtube-emotion-distilbert</t>
+          <t>https://www.youtube.com/watch?v=M8To7iorkxQ</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>150 reviewed Streamlit app comments</t>
+          <t>Pre-tuning baseline</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>CPU</t>
-        </is>
-      </c>
-      <c r="D3" s="2" t="n">
-        <v>150</v>
+          <t>j-hartmann/emotion-english-distilroberta-base</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>7-emotion</t>
+        </is>
       </c>
       <c r="E3" s="2" t="n">
-        <v>12.8617</v>
+        <v>26</v>
       </c>
       <c r="F3" s="2" t="n">
-        <v>1.3363</v>
-      </c>
-      <c r="G3" s="2" t="inlineStr">
-        <is>
-          <t>GoEmotions fine-tuned DistilBERT</t>
-        </is>
+        <v>50</v>
+      </c>
+      <c r="G3" s="2" t="n">
+        <v>0.52</v>
+      </c>
+      <c r="H3" s="2" t="n">
+        <v>1.48</v>
+      </c>
+      <c r="I3" s="2" t="n">
+        <v>1.52</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>chase1zhang/youtube-emotion-distilbert-domain-adapted</t>
+          <t>https://www.youtube.com/watch?v=-_-eIVAX1yQ</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>150 reviewed Streamlit app comments</t>
+          <t>Pre-tuning baseline</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>CPU</t>
-        </is>
-      </c>
-      <c r="D4" s="2" t="n">
-        <v>150</v>
+          <t>j-hartmann/emotion-english-distilroberta-base</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>7-emotion</t>
+        </is>
       </c>
       <c r="E4" s="2" t="n">
-        <v>14.8326</v>
+        <v>12</v>
       </c>
       <c r="F4" s="2" t="n">
-        <v>1.4346</v>
-      </c>
-      <c r="G4" s="2" t="inlineStr">
-        <is>
-          <t>YouTube-domain adapted DistilBERT</t>
-        </is>
+        <v>50</v>
+      </c>
+      <c r="G4" s="2" t="n">
+        <v>0.24</v>
+      </c>
+      <c r="H4" s="2" t="n">
+        <v>1.48</v>
+      </c>
+      <c r="I4" s="2" t="n">
+        <v>1.52</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>SamLowe/roberta-base-go_emotions</t>
+          <t>OVERALL</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>150 reviewed Streamlit app comments</t>
+          <t>Pre-tuning baseline</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>CPU</t>
-        </is>
-      </c>
-      <c r="D5" s="2" t="n">
+          <t>j-hartmann/emotion-english-distilroberta-base</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>7-emotion</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="n">
+        <v>67</v>
+      </c>
+      <c r="F5" s="2" t="n">
         <v>150</v>
       </c>
-      <c r="E5" s="2" t="n">
-        <v>4.8483</v>
-      </c>
-      <c r="F5" s="2" t="n">
-        <v>3.8838</v>
-      </c>
-      <c r="G5" s="2" t="inlineStr">
-        <is>
-          <t>public GoEmotions RoBERTa</t>
-        </is>
+      <c r="G5" s="2" t="n">
+        <v>0.4466666666666666</v>
+      </c>
+      <c r="H5" s="2" t="n">
+        <v>1.48</v>
+      </c>
+      <c r="I5" s="2" t="n">
+        <v>1.52</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>j-hartmann/emotion-english-roberta-large</t>
+          <t>https://www.youtube.com/watch?v=d2dgJGkw5p0</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>150 reviewed Streamlit app comments</t>
+          <t>GoEmotions fine-tuned</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>CPU</t>
-        </is>
-      </c>
-      <c r="D6" s="2" t="n">
-        <v>150</v>
+          <t>chase1zhang/youtube-emotion-distilbert</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>7-emotion</t>
+        </is>
       </c>
       <c r="E6" s="2" t="n">
-        <v>40.846</v>
+        <v>29</v>
       </c>
       <c r="F6" s="2" t="n">
-        <v>11.9566</v>
-      </c>
-      <c r="G6" s="2" t="inlineStr">
-        <is>
-          <t>public RoBERTa-large seven-emotion</t>
-        </is>
+        <v>50</v>
+      </c>
+      <c r="G6" s="2" t="n">
+        <v>0.58</v>
+      </c>
+      <c r="H6" s="2" t="n">
+        <v>0.82</v>
+      </c>
+      <c r="I6" s="2" t="n">
+        <v>1.88</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
+          <t>https://www.youtube.com/watch?v=M8To7iorkxQ</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>GoEmotions fine-tuned</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>chase1zhang/youtube-emotion-distilbert</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>7-emotion</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="n">
+        <v>25</v>
+      </c>
+      <c r="F7" s="2" t="n">
+        <v>50</v>
+      </c>
+      <c r="G7" s="2" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="H7" s="2" t="n">
+        <v>0.82</v>
+      </c>
+      <c r="I7" s="2" t="n">
+        <v>1.88</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=-_-eIVAX1yQ</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>GoEmotions fine-tuned</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>chase1zhang/youtube-emotion-distilbert</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>7-emotion</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="n">
+        <v>16</v>
+      </c>
+      <c r="F8" s="2" t="n">
+        <v>50</v>
+      </c>
+      <c r="G8" s="2" t="n">
+        <v>0.32</v>
+      </c>
+      <c r="H8" s="2" t="n">
+        <v>0.82</v>
+      </c>
+      <c r="I8" s="2" t="n">
+        <v>1.88</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>OVERALL</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>GoEmotions fine-tuned</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>chase1zhang/youtube-emotion-distilbert</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>7-emotion</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="n">
+        <v>70</v>
+      </c>
+      <c r="F9" s="2" t="n">
+        <v>150</v>
+      </c>
+      <c r="G9" s="2" t="n">
+        <v>0.4666666666666667</v>
+      </c>
+      <c r="H9" s="2" t="n">
+        <v>0.82</v>
+      </c>
+      <c r="I9" s="2" t="n">
+        <v>1.88</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=d2dgJGkw5p0</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>YouTube-domain adapted (your model)</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>chase1zhang/youtube-emotion-distilbert-domain-adapted</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>7-emotion</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="n">
+        <v>28</v>
+      </c>
+      <c r="F10" s="2" t="n">
+        <v>50</v>
+      </c>
+      <c r="G10" s="2" t="n">
+        <v>0.5600000000000001</v>
+      </c>
+      <c r="H10" s="2" t="n">
+        <v>0.82</v>
+      </c>
+      <c r="I10" s="2" t="n">
+        <v>1.84</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=M8To7iorkxQ</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>YouTube-domain adapted (your model)</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>chase1zhang/youtube-emotion-distilbert-domain-adapted</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>7-emotion</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="n">
+        <v>25</v>
+      </c>
+      <c r="F11" s="2" t="n">
+        <v>50</v>
+      </c>
+      <c r="G11" s="2" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="H11" s="2" t="n">
+        <v>0.82</v>
+      </c>
+      <c r="I11" s="2" t="n">
+        <v>1.84</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=-_-eIVAX1yQ</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>YouTube-domain adapted (your model)</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>chase1zhang/youtube-emotion-distilbert-domain-adapted</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>7-emotion</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="n">
+        <v>18</v>
+      </c>
+      <c r="F12" s="2" t="n">
+        <v>50</v>
+      </c>
+      <c r="G12" s="2" t="n">
+        <v>0.36</v>
+      </c>
+      <c r="H12" s="2" t="n">
+        <v>0.82</v>
+      </c>
+      <c r="I12" s="2" t="n">
+        <v>1.84</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>OVERALL</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>YouTube-domain adapted (your model)</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>chase1zhang/youtube-emotion-distilbert-domain-adapted</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>7-emotion</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="n">
+        <v>71</v>
+      </c>
+      <c r="F13" s="2" t="n">
+        <v>150</v>
+      </c>
+      <c r="G13" s="2" t="n">
+        <v>0.4733333333333333</v>
+      </c>
+      <c r="H13" s="2" t="n">
+        <v>0.82</v>
+      </c>
+      <c r="I13" s="2" t="n">
+        <v>1.84</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=d2dgJGkw5p0</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>Public GoEmotions RoBERTa (SamLowe)</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>SamLowe/roberta-base-go_emotions</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>7-emotion</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="n">
+        <v>21</v>
+      </c>
+      <c r="F14" s="2" t="n">
+        <v>50</v>
+      </c>
+      <c r="G14" s="2" t="n">
+        <v>0.42</v>
+      </c>
+      <c r="H14" s="2" t="n">
+        <v>0.84</v>
+      </c>
+      <c r="I14" s="2" t="n">
+        <v>4.01</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=M8To7iorkxQ</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>Public GoEmotions RoBERTa (SamLowe)</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>SamLowe/roberta-base-go_emotions</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>7-emotion</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="F15" s="2" t="n">
+        <v>50</v>
+      </c>
+      <c r="G15" s="2" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="H15" s="2" t="n">
+        <v>0.84</v>
+      </c>
+      <c r="I15" s="2" t="n">
+        <v>4.01</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=-_-eIVAX1yQ</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>Public GoEmotions RoBERTa (SamLowe)</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>SamLowe/roberta-base-go_emotions</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>7-emotion</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="F16" s="2" t="n">
+        <v>50</v>
+      </c>
+      <c r="G16" s="2" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="H16" s="2" t="n">
+        <v>0.84</v>
+      </c>
+      <c r="I16" s="2" t="n">
+        <v>4.01</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>OVERALL</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>Public GoEmotions RoBERTa (SamLowe)</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>SamLowe/roberta-base-go_emotions</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>7-emotion</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="n">
+        <v>41</v>
+      </c>
+      <c r="F17" s="2" t="n">
+        <v>150</v>
+      </c>
+      <c r="G17" s="2" t="n">
+        <v>0.2733333333333333</v>
+      </c>
+      <c r="H17" s="2" t="n">
+        <v>0.84</v>
+      </c>
+      <c r="I17" s="2" t="n">
+        <v>4.01</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=d2dgJGkw5p0</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>Public RoBERTa-large 7-emotion</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>j-hartmann/emotion-english-roberta-large</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>7-emotion</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="n">
+        <v>24</v>
+      </c>
+      <c r="F18" s="2" t="n">
+        <v>50</v>
+      </c>
+      <c r="G18" s="2" t="n">
+        <v>0.48</v>
+      </c>
+      <c r="H18" s="2" t="n">
+        <v>1.73</v>
+      </c>
+      <c r="I18" s="2" t="n">
+        <v>9.51</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=M8To7iorkxQ</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>Public RoBERTa-large 7-emotion</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>j-hartmann/emotion-english-roberta-large</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>7-emotion</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="n">
+        <v>24</v>
+      </c>
+      <c r="F19" s="2" t="n">
+        <v>50</v>
+      </c>
+      <c r="G19" s="2" t="n">
+        <v>0.48</v>
+      </c>
+      <c r="H19" s="2" t="n">
+        <v>1.73</v>
+      </c>
+      <c r="I19" s="2" t="n">
+        <v>9.51</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=-_-eIVAX1yQ</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>Public RoBERTa-large 7-emotion</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>j-hartmann/emotion-english-roberta-large</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>7-emotion</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="n">
+        <v>14</v>
+      </c>
+      <c r="F20" s="2" t="n">
+        <v>50</v>
+      </c>
+      <c r="G20" s="2" t="n">
+        <v>0.28</v>
+      </c>
+      <c r="H20" s="2" t="n">
+        <v>1.73</v>
+      </c>
+      <c r="I20" s="2" t="n">
+        <v>9.51</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>OVERALL</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>Public RoBERTa-large 7-emotion</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>j-hartmann/emotion-english-roberta-large</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>7-emotion</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="n">
+        <v>62</v>
+      </c>
+      <c r="F21" s="2" t="n">
+        <v>150</v>
+      </c>
+      <c r="G21" s="2" t="n">
+        <v>0.4133333333333333</v>
+      </c>
+      <c r="H21" s="2" t="n">
+        <v>1.73</v>
+      </c>
+      <c r="I21" s="2" t="n">
+        <v>9.51</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>OVERALL</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>3-sentiment pipeline</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
           <t>cardiffnlp/twitter-roberta-base-sentiment-latest</t>
         </is>
       </c>
-      <c r="B7" s="2" t="inlineStr">
-        <is>
-          <t>150 reviewed Streamlit app comments</t>
-        </is>
-      </c>
-      <c r="C7" s="2" t="inlineStr">
-        <is>
-          <t>CPU</t>
-        </is>
-      </c>
-      <c r="D7" s="2" t="n">
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>3-sentiment</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="n">
+        <v>105</v>
+      </c>
+      <c r="F22" s="2" t="n">
         <v>150</v>
       </c>
-      <c r="E7" s="2" t="n">
-        <v>4.304</v>
-      </c>
-      <c r="F7" s="2" t="n">
-        <v>3.0499</v>
-      </c>
-      <c r="G7" s="2" t="inlineStr">
-        <is>
-          <t>supporting sentiment pipeline</t>
-        </is>
+      <c r="G22" s="2" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="H22" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I22" s="2" t="n">
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -1768,13 +2372,259 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:G7"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="45" customWidth="1" min="1" max="1"/>
+    <col width="37" customWidth="1" min="2" max="2"/>
+    <col width="8" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="36" customWidth="1" min="5" max="5"/>
+    <col width="39" customWidth="1" min="6" max="6"/>
+    <col width="36" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>model_name</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>dataset</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>device</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>num_comments</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>runtime_with_model_loading_seconds</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>runtime_without_model_loading_seconds</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>j-hartmann/emotion-english-distilroberta-base</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>150 reviewed Streamlit app comments</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>CPU</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="n">
+        <v>150</v>
+      </c>
+      <c r="E2" s="2" t="n">
+        <v>7.2815</v>
+      </c>
+      <c r="F2" s="2" t="n">
+        <v>1.5164</v>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>pre-tuning public baseline</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>chase1zhang/youtube-emotion-distilbert</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>150 reviewed Streamlit app comments</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>CPU</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="n">
+        <v>150</v>
+      </c>
+      <c r="E3" s="2" t="n">
+        <v>12.8617</v>
+      </c>
+      <c r="F3" s="2" t="n">
+        <v>1.3363</v>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>GoEmotions fine-tuned DistilBERT</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>chase1zhang/youtube-emotion-distilbert-domain-adapted</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>150 reviewed Streamlit app comments</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>CPU</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="n">
+        <v>150</v>
+      </c>
+      <c r="E4" s="2" t="n">
+        <v>14.8326</v>
+      </c>
+      <c r="F4" s="2" t="n">
+        <v>1.4346</v>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>YouTube-domain adapted DistilBERT</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>SamLowe/roberta-base-go_emotions</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>150 reviewed Streamlit app comments</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>CPU</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="n">
+        <v>150</v>
+      </c>
+      <c r="E5" s="2" t="n">
+        <v>4.8483</v>
+      </c>
+      <c r="F5" s="2" t="n">
+        <v>3.8838</v>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>public GoEmotions RoBERTa</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>j-hartmann/emotion-english-roberta-large</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>150 reviewed Streamlit app comments</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>CPU</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="n">
+        <v>150</v>
+      </c>
+      <c r="E6" s="2" t="n">
+        <v>40.846</v>
+      </c>
+      <c r="F6" s="2" t="n">
+        <v>11.9566</v>
+      </c>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>public RoBERTa-large seven-emotion</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>cardiffnlp/twitter-roberta-base-sentiment-latest</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>150 reviewed Streamlit app comments</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>CPU</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="n">
+        <v>150</v>
+      </c>
+      <c r="E7" s="2" t="n">
+        <v>4.304</v>
+      </c>
+      <c r="F7" s="2" t="n">
+        <v>3.0499</v>
+      </c>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>supporting sentiment pipeline</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:H151"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="40" customWidth="1" min="1" max="1"/>
+    <col width="45" customWidth="1" min="1" max="1"/>
     <col width="15" customWidth="1" min="2" max="2"/>
     <col width="15" customWidth="1" min="3" max="3"/>
-    <col width="40" customWidth="1" min="4" max="4"/>
+    <col width="45" customWidth="1" min="4" max="4"/>
     <col width="18" customWidth="1" min="5" max="5"/>
     <col width="20" customWidth="1" min="6" max="6"/>
     <col width="26" customWidth="1" min="7" max="7"/>

</xml_diff>

<commit_message>
Clean up experiments and notebooks, update xlsx with latest results
- Deleted 4 intermediate CSV files from experiments/ (data now in xlsx)
- Deleted 2 CSV result files from notebooks/ (no longer needed)
- Updated Experimental_results.xlsx with latest Colab notebook results
- Kept: Experimental_results.xlsx, Performance_result.xlsx, app_per_comment_manual_labels.csv

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/experiments/Experimental_results.xlsx
+++ b/experiments/Experimental_results.xlsx
@@ -1,19 +1,19 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Model_Selection" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="YouTube_Domain_Validation" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Streamlit_App_Performance" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="App_5Model_Comparison" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="App_Runtime" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Model_Revisions" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Manual_Comment_Labels" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Model_Selection" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="YouTube_Domain_Validation" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Streamlit_App_Performance" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="App_5Model_Comparison" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="App_Runtime" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Model_Revisions" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Manual_Comment_Labels" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1526,10 +1526,10 @@
         <v>50</v>
       </c>
       <c r="F5" t="n">
-        <v>24</v>
+        <v>29</v>
       </c>
       <c r="G5" t="n">
-        <v>0.48</v>
+        <v>0.58</v>
       </c>
       <c r="H5" t="inlineStr">
         <is>
@@ -1577,10 +1577,10 @@
         <v>50</v>
       </c>
       <c r="F6" t="n">
-        <v>17</v>
+        <v>25</v>
       </c>
       <c r="G6" t="n">
-        <v>0.34</v>
+        <v>0.5</v>
       </c>
       <c r="H6" t="inlineStr">
         <is>
@@ -1628,10 +1628,10 @@
         <v>50</v>
       </c>
       <c r="F7" t="n">
-        <v>8</v>
+        <v>16</v>
       </c>
       <c r="G7" t="n">
-        <v>0.16</v>
+        <v>0.32</v>
       </c>
       <c r="H7" t="inlineStr">
         <is>
@@ -1679,10 +1679,10 @@
         <v>50</v>
       </c>
       <c r="F8" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="G8" t="n">
-        <v>0.54</v>
+        <v>0.5600000000000001</v>
       </c>
       <c r="H8" t="inlineStr">
         <is>
@@ -1730,10 +1730,10 @@
         <v>50</v>
       </c>
       <c r="F9" t="n">
-        <v>33</v>
+        <v>25</v>
       </c>
       <c r="G9" t="n">
-        <v>0.66</v>
+        <v>0.5</v>
       </c>
       <c r="H9" t="inlineStr">
         <is>
@@ -1781,10 +1781,10 @@
         <v>50</v>
       </c>
       <c r="F10" t="n">
-        <v>24</v>
+        <v>18</v>
       </c>
       <c r="G10" t="n">
-        <v>0.48</v>
+        <v>0.36</v>
       </c>
       <c r="H10" t="inlineStr">
         <is>
@@ -1832,10 +1832,10 @@
         <v>50</v>
       </c>
       <c r="F11" t="n">
-        <v>26</v>
+        <v>21</v>
       </c>
       <c r="G11" t="n">
-        <v>0.52</v>
+        <v>0.42</v>
       </c>
       <c r="H11" t="inlineStr">
         <is>
@@ -1883,10 +1883,10 @@
         <v>50</v>
       </c>
       <c r="F12" t="n">
-        <v>37</v>
+        <v>10</v>
       </c>
       <c r="G12" t="n">
-        <v>0.74</v>
+        <v>0.2</v>
       </c>
       <c r="H12" t="inlineStr">
         <is>
@@ -1934,10 +1934,10 @@
         <v>50</v>
       </c>
       <c r="F13" t="n">
-        <v>17</v>
+        <v>10</v>
       </c>
       <c r="G13" t="n">
-        <v>0.34</v>
+        <v>0.2</v>
       </c>
       <c r="H13" t="inlineStr">
         <is>
@@ -3107,10 +3107,10 @@
         <v>150</v>
       </c>
       <c r="F36" t="n">
-        <v>49</v>
+        <v>70</v>
       </c>
       <c r="G36" t="n">
-        <v>0.3267</v>
+        <v>0.4667</v>
       </c>
       <c r="H36" t="inlineStr">
         <is>
@@ -3158,10 +3158,10 @@
         <v>150</v>
       </c>
       <c r="F37" t="n">
-        <v>84</v>
+        <v>71</v>
       </c>
       <c r="G37" t="n">
-        <v>0.5600000000000001</v>
+        <v>0.4733</v>
       </c>
       <c r="H37" t="inlineStr">
         <is>
@@ -3209,10 +3209,10 @@
         <v>150</v>
       </c>
       <c r="F38" t="n">
-        <v>80</v>
+        <v>41</v>
       </c>
       <c r="G38" t="n">
-        <v>0.5333</v>
+        <v>0.2733</v>
       </c>
       <c r="H38" t="inlineStr">
         <is>
@@ -3603,7 +3603,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I45"/>
+  <dimension ref="A1:I19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3683,27 +3683,21 @@
       <c r="G2" t="n">
         <v>0.58</v>
       </c>
-      <c r="H2" t="n">
-        <v>1.2324</v>
-      </c>
-      <c r="I2" t="n">
-        <v>1.0282</v>
-      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=M8To7iorkxQ</t>
+          <t>https://www.youtube.com/watch?v=d2dgJGkw5p0</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Pre-tuning baseline</t>
+          <t>GoEmotions fine-tuned</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>j-hartmann/emotion-english-distilroberta-base</t>
+          <t>chase1zhang/youtube-emotion-distilbert</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -3712,35 +3706,29 @@
         </is>
       </c>
       <c r="E3" t="n">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="F3" t="n">
         <v>50</v>
       </c>
       <c r="G3" t="n">
-        <v>0.52</v>
-      </c>
-      <c r="H3" t="n">
-        <v>1.2324</v>
-      </c>
-      <c r="I3" t="n">
-        <v>1.0282</v>
+        <v>0.58</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=-_-eIVAX1yQ</t>
+          <t>https://www.youtube.com/watch?v=d2dgJGkw5p0</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Pre-tuning baseline</t>
+          <t>YouTube-domain adapted</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>j-hartmann/emotion-english-distilroberta-base</t>
+          <t>chase1zhang/youtube-emotion-distilbert-domain-adapted</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -3749,19 +3737,13 @@
         </is>
       </c>
       <c r="E4" t="n">
-        <v>12</v>
+        <v>28</v>
       </c>
       <c r="F4" t="n">
         <v>50</v>
       </c>
       <c r="G4" t="n">
-        <v>0.24</v>
-      </c>
-      <c r="H4" t="n">
-        <v>1.2324</v>
-      </c>
-      <c r="I4" t="n">
-        <v>1.0282</v>
+        <v>0.5600000000000001</v>
       </c>
     </row>
     <row r="5">
@@ -3772,12 +3754,12 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>GoEmotions fine-tuned</t>
+          <t>Public RoBERTa-large</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>chase1zhang/youtube-emotion-distilbert</t>
+          <t>j-hartmann/emotion-english-roberta-large</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -3793,28 +3775,22 @@
       </c>
       <c r="G5" t="n">
         <v>0.48</v>
-      </c>
-      <c r="H5" t="n">
-        <v>0.0582</v>
-      </c>
-      <c r="I5" t="n">
-        <v>0.8488</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=M8To7iorkxQ</t>
+          <t>https://www.youtube.com/watch?v=d2dgJGkw5p0</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>GoEmotions fine-tuned</t>
+          <t>Public GoEmotions RoBERTa</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>chase1zhang/youtube-emotion-distilbert</t>
+          <t>SamLowe/roberta-base-go_emotions</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -3823,72 +3799,60 @@
         </is>
       </c>
       <c r="E6" t="n">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="F6" t="n">
         <v>50</v>
       </c>
       <c r="G6" t="n">
-        <v>0.34</v>
-      </c>
-      <c r="H6" t="n">
-        <v>0.0582</v>
-      </c>
-      <c r="I6" t="n">
-        <v>0.8488</v>
+        <v>0.42</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=-_-eIVAX1yQ</t>
+          <t>https://www.youtube.com/watch?v=d2dgJGkw5p0</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>GoEmotions fine-tuned</t>
+          <t>Sentiment pipeline</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>chase1zhang/youtube-emotion-distilbert</t>
+          <t>cardiffnlp/twitter-roberta-base-sentiment-latest</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>7-emotion</t>
+          <t>3-sentiment</t>
         </is>
       </c>
       <c r="E7" t="n">
-        <v>8</v>
+        <v>30</v>
       </c>
       <c r="F7" t="n">
         <v>50</v>
       </c>
       <c r="G7" t="n">
-        <v>0.16</v>
-      </c>
-      <c r="H7" t="n">
-        <v>0.0582</v>
-      </c>
-      <c r="I7" t="n">
-        <v>0.8488</v>
+        <v>0.6</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=d2dgJGkw5p0</t>
+          <t>https://www.youtube.com/watch?v=M8To7iorkxQ</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>YouTube-domain adapted (your model)</t>
+          <t>Pre-tuning baseline</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>chase1zhang/youtube-emotion-distilbert-domain-adapted</t>
+          <t>j-hartmann/emotion-english-distilroberta-base</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -3897,19 +3861,13 @@
         </is>
       </c>
       <c r="E8" t="n">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="F8" t="n">
         <v>50</v>
       </c>
       <c r="G8" t="n">
-        <v>0.54</v>
-      </c>
-      <c r="H8" t="n">
-        <v>0.0385</v>
-      </c>
-      <c r="I8" t="n">
-        <v>0.9343</v>
+        <v>0.52</v>
       </c>
     </row>
     <row r="9">
@@ -3920,12 +3878,12 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>YouTube-domain adapted (your model)</t>
+          <t>GoEmotions fine-tuned</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>chase1zhang/youtube-emotion-distilbert-domain-adapted</t>
+          <t>chase1zhang/youtube-emotion-distilbert</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -3934,30 +3892,24 @@
         </is>
       </c>
       <c r="E9" t="n">
-        <v>33</v>
+        <v>25</v>
       </c>
       <c r="F9" t="n">
         <v>50</v>
       </c>
       <c r="G9" t="n">
-        <v>0.66</v>
-      </c>
-      <c r="H9" t="n">
-        <v>0.0385</v>
-      </c>
-      <c r="I9" t="n">
-        <v>0.9343</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=-_-eIVAX1yQ</t>
+          <t>https://www.youtube.com/watch?v=M8To7iorkxQ</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>YouTube-domain adapted (your model)</t>
+          <t>YouTube-domain adapted</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -3971,35 +3923,29 @@
         </is>
       </c>
       <c r="E10" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="F10" t="n">
         <v>50</v>
       </c>
       <c r="G10" t="n">
-        <v>0.48</v>
-      </c>
-      <c r="H10" t="n">
-        <v>0.0385</v>
-      </c>
-      <c r="I10" t="n">
-        <v>0.9343</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=d2dgJGkw5p0</t>
+          <t>https://www.youtube.com/watch?v=M8To7iorkxQ</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Public GoEmotions RoBERTa (SamLowe)</t>
+          <t>Public RoBERTa-large</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>SamLowe/roberta-base-go_emotions</t>
+          <t>j-hartmann/emotion-english-roberta-large</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -4008,19 +3954,13 @@
         </is>
       </c>
       <c r="E11" t="n">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="F11" t="n">
         <v>50</v>
       </c>
       <c r="G11" t="n">
-        <v>0.52</v>
-      </c>
-      <c r="H11" t="n">
-        <v>0.9086</v>
-      </c>
-      <c r="I11" t="n">
-        <v>1.8941</v>
+        <v>0.48</v>
       </c>
     </row>
     <row r="12">
@@ -4031,7 +3971,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Public GoEmotions RoBERTa (SamLowe)</t>
+          <t>Public GoEmotions RoBERTa</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -4045,72 +3985,60 @@
         </is>
       </c>
       <c r="E12" t="n">
-        <v>37</v>
+        <v>10</v>
       </c>
       <c r="F12" t="n">
         <v>50</v>
       </c>
       <c r="G12" t="n">
-        <v>0.74</v>
-      </c>
-      <c r="H12" t="n">
-        <v>0.9086</v>
-      </c>
-      <c r="I12" t="n">
-        <v>1.8941</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=-_-eIVAX1yQ</t>
+          <t>https://www.youtube.com/watch?v=M8To7iorkxQ</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Public GoEmotions RoBERTa (SamLowe)</t>
+          <t>Sentiment pipeline</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>SamLowe/roberta-base-go_emotions</t>
+          <t>cardiffnlp/twitter-roberta-base-sentiment-latest</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>7-emotion</t>
+          <t>3-sentiment</t>
         </is>
       </c>
       <c r="E13" t="n">
-        <v>17</v>
+        <v>46</v>
       </c>
       <c r="F13" t="n">
         <v>50</v>
       </c>
       <c r="G13" t="n">
-        <v>0.34</v>
-      </c>
-      <c r="H13" t="n">
-        <v>0.9086</v>
-      </c>
-      <c r="I13" t="n">
-        <v>1.8941</v>
+        <v>0.92</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=d2dgJGkw5p0</t>
+          <t>https://www.youtube.com/watch?v=-_-eIVAX1yQ</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Public RoBERTa-large 7-emotion</t>
+          <t>Pre-tuning baseline</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>j-hartmann/emotion-english-roberta-large</t>
+          <t>j-hartmann/emotion-english-distilroberta-base</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -4119,35 +4047,29 @@
         </is>
       </c>
       <c r="E14" t="n">
-        <v>24</v>
+        <v>12</v>
       </c>
       <c r="F14" t="n">
         <v>50</v>
       </c>
       <c r="G14" t="n">
-        <v>0.48</v>
-      </c>
-      <c r="H14" t="n">
-        <v>1.4107</v>
-      </c>
-      <c r="I14" t="n">
-        <v>7.1657</v>
+        <v>0.24</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=M8To7iorkxQ</t>
+          <t>https://www.youtube.com/watch?v=-_-eIVAX1yQ</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Public RoBERTa-large 7-emotion</t>
+          <t>GoEmotions fine-tuned</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>j-hartmann/emotion-english-roberta-large</t>
+          <t>chase1zhang/youtube-emotion-distilbert</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -4156,19 +4078,13 @@
         </is>
       </c>
       <c r="E15" t="n">
-        <v>24</v>
+        <v>16</v>
       </c>
       <c r="F15" t="n">
         <v>50</v>
       </c>
       <c r="G15" t="n">
-        <v>0.48</v>
-      </c>
-      <c r="H15" t="n">
-        <v>1.4107</v>
-      </c>
-      <c r="I15" t="n">
-        <v>7.1657</v>
+        <v>0.32</v>
       </c>
     </row>
     <row r="16">
@@ -4179,12 +4095,12 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Public RoBERTa-large 7-emotion</t>
+          <t>YouTube-domain adapted</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>j-hartmann/emotion-english-roberta-large</t>
+          <t>chase1zhang/youtube-emotion-distilbert-domain-adapted</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -4193,35 +4109,29 @@
         </is>
       </c>
       <c r="E16" t="n">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="F16" t="n">
         <v>50</v>
       </c>
       <c r="G16" t="n">
-        <v>0.28</v>
-      </c>
-      <c r="H16" t="n">
-        <v>1.4107</v>
-      </c>
-      <c r="I16" t="n">
-        <v>7.1657</v>
+        <v>0.36</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=d2dgJGkw5p0</t>
+          <t>https://www.youtube.com/watch?v=-_-eIVAX1yQ</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>YouTube-domain adapted RoBERTa (SamLowe)</t>
+          <t>Public RoBERTa-large</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>chase1zhang/youtube-emotion-samlowe-roberta-domain-adapted</t>
+          <t>j-hartmann/emotion-english-roberta-large</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -4230,35 +4140,29 @@
         </is>
       </c>
       <c r="E17" t="n">
-        <v>30</v>
+        <v>14</v>
       </c>
       <c r="F17" t="n">
         <v>50</v>
       </c>
       <c r="G17" t="n">
-        <v>0.6</v>
-      </c>
-      <c r="H17" t="n">
-        <v>0.1597</v>
-      </c>
-      <c r="I17" t="n">
-        <v>2.0179</v>
+        <v>0.28</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=M8To7iorkxQ</t>
+          <t>https://www.youtube.com/watch?v=-_-eIVAX1yQ</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>YouTube-domain adapted RoBERTa (SamLowe)</t>
+          <t>Public GoEmotions RoBERTa</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>chase1zhang/youtube-emotion-samlowe-roberta-domain-adapted</t>
+          <t>SamLowe/roberta-base-go_emotions</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -4267,19 +4171,13 @@
         </is>
       </c>
       <c r="E18" t="n">
-        <v>42</v>
+        <v>10</v>
       </c>
       <c r="F18" t="n">
         <v>50</v>
       </c>
       <c r="G18" t="n">
-        <v>0.84</v>
-      </c>
-      <c r="H18" t="n">
-        <v>0.1597</v>
-      </c>
-      <c r="I18" t="n">
-        <v>2.0179</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="19">
@@ -4290,995 +4188,27 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>YouTube-domain adapted RoBERTa (SamLowe)</t>
+          <t>Sentiment pipeline</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>chase1zhang/youtube-emotion-samlowe-roberta-domain-adapted</t>
+          <t>cardiffnlp/twitter-roberta-base-sentiment-latest</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>7-emotion</t>
+          <t>3-sentiment</t>
         </is>
       </c>
       <c r="E19" t="n">
-        <v>21</v>
+        <v>29</v>
       </c>
       <c r="F19" t="n">
         <v>50</v>
       </c>
       <c r="G19" t="n">
-        <v>0.42</v>
-      </c>
-      <c r="H19" t="n">
-        <v>0.1597</v>
-      </c>
-      <c r="I19" t="n">
-        <v>2.0179</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=d2dgJGkw5p0</t>
-        </is>
-      </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>YouTube-domain adapted DistilRoBERTa (j-hartmann)</t>
-        </is>
-      </c>
-      <c r="C20" t="inlineStr">
-        <is>
-          <t>chase1zhang/youtube-emotion-jhartmann-distilroberta-domain-adapted</t>
-        </is>
-      </c>
-      <c r="D20" t="inlineStr">
-        <is>
-          <t>7-emotion</t>
-        </is>
-      </c>
-      <c r="E20" t="n">
-        <v>25</v>
-      </c>
-      <c r="F20" t="n">
-        <v>50</v>
-      </c>
-      <c r="G20" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="H20" t="n">
-        <v>0.0912</v>
-      </c>
-      <c r="I20" t="n">
-        <v>1.0381</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=M8To7iorkxQ</t>
-        </is>
-      </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>YouTube-domain adapted DistilRoBERTa (j-hartmann)</t>
-        </is>
-      </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>chase1zhang/youtube-emotion-jhartmann-distilroberta-domain-adapted</t>
-        </is>
-      </c>
-      <c r="D21" t="inlineStr">
-        <is>
-          <t>7-emotion</t>
-        </is>
-      </c>
-      <c r="E21" t="n">
-        <v>36</v>
-      </c>
-      <c r="F21" t="n">
-        <v>50</v>
-      </c>
-      <c r="G21" t="n">
-        <v>0.72</v>
-      </c>
-      <c r="H21" t="n">
-        <v>0.0912</v>
-      </c>
-      <c r="I21" t="n">
-        <v>1.0381</v>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=-_-eIVAX1yQ</t>
-        </is>
-      </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>YouTube-domain adapted DistilRoBERTa (j-hartmann)</t>
-        </is>
-      </c>
-      <c r="C22" t="inlineStr">
-        <is>
-          <t>chase1zhang/youtube-emotion-jhartmann-distilroberta-domain-adapted</t>
-        </is>
-      </c>
-      <c r="D22" t="inlineStr">
-        <is>
-          <t>7-emotion</t>
-        </is>
-      </c>
-      <c r="E22" t="n">
-        <v>22</v>
-      </c>
-      <c r="F22" t="n">
-        <v>50</v>
-      </c>
-      <c r="G22" t="n">
-        <v>0.44</v>
-      </c>
-      <c r="H22" t="n">
-        <v>0.0912</v>
-      </c>
-      <c r="I22" t="n">
-        <v>1.0381</v>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=d2dgJGkw5p0</t>
-        </is>
-      </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>YouTube-domain adapted RoBERTa-large (j-hartmann)</t>
-        </is>
-      </c>
-      <c r="C23" t="inlineStr">
-        <is>
-          <t>chase1zhang/youtube-emotion-roberta-large-domain-adapted</t>
-        </is>
-      </c>
-      <c r="D23" t="inlineStr">
-        <is>
-          <t>7-emotion</t>
-        </is>
-      </c>
-      <c r="E23" t="n">
-        <v>30</v>
-      </c>
-      <c r="F23" t="n">
-        <v>50</v>
-      </c>
-      <c r="G23" t="n">
-        <v>0.6</v>
-      </c>
-      <c r="H23" t="n">
-        <v>0.186</v>
-      </c>
-      <c r="I23" t="n">
-        <v>7.3825</v>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=M8To7iorkxQ</t>
-        </is>
-      </c>
-      <c r="B24" t="inlineStr">
-        <is>
-          <t>YouTube-domain adapted RoBERTa-large (j-hartmann)</t>
-        </is>
-      </c>
-      <c r="C24" t="inlineStr">
-        <is>
-          <t>chase1zhang/youtube-emotion-roberta-large-domain-adapted</t>
-        </is>
-      </c>
-      <c r="D24" t="inlineStr">
-        <is>
-          <t>7-emotion</t>
-        </is>
-      </c>
-      <c r="E24" t="n">
-        <v>43</v>
-      </c>
-      <c r="F24" t="n">
-        <v>50</v>
-      </c>
-      <c r="G24" t="n">
-        <v>0.86</v>
-      </c>
-      <c r="H24" t="n">
-        <v>0.186</v>
-      </c>
-      <c r="I24" t="n">
-        <v>7.3825</v>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=-_-eIVAX1yQ</t>
-        </is>
-      </c>
-      <c r="B25" t="inlineStr">
-        <is>
-          <t>YouTube-domain adapted RoBERTa-large (j-hartmann)</t>
-        </is>
-      </c>
-      <c r="C25" t="inlineStr">
-        <is>
-          <t>chase1zhang/youtube-emotion-roberta-large-domain-adapted</t>
-        </is>
-      </c>
-      <c r="D25" t="inlineStr">
-        <is>
-          <t>7-emotion</t>
-        </is>
-      </c>
-      <c r="E25" t="n">
-        <v>21</v>
-      </c>
-      <c r="F25" t="n">
-        <v>50</v>
-      </c>
-      <c r="G25" t="n">
-        <v>0.42</v>
-      </c>
-      <c r="H25" t="n">
-        <v>0.186</v>
-      </c>
-      <c r="I25" t="n">
-        <v>7.3825</v>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=d2dgJGkw5p0</t>
-        </is>
-      </c>
-      <c r="B26" t="inlineStr">
-        <is>
-          <t>CardiffNLP Twitter RoBERTa</t>
-        </is>
-      </c>
-      <c r="C26" t="inlineStr">
-        <is>
-          <t>cardiffnlp/twitter-roberta-base-sentiment-latest</t>
-        </is>
-      </c>
-      <c r="D26" t="inlineStr">
-        <is>
-          <t>3-sentiment</t>
-        </is>
-      </c>
-      <c r="E26" t="n">
-        <v>30</v>
-      </c>
-      <c r="F26" t="n">
-        <v>50</v>
-      </c>
-      <c r="G26" t="n">
-        <v>0.6</v>
-      </c>
-      <c r="H26" t="n">
-        <v>1.2355</v>
-      </c>
-      <c r="I26" t="n">
-        <v>2.0197</v>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=M8To7iorkxQ</t>
-        </is>
-      </c>
-      <c r="B27" t="inlineStr">
-        <is>
-          <t>CardiffNLP Twitter RoBERTa</t>
-        </is>
-      </c>
-      <c r="C27" t="inlineStr">
-        <is>
-          <t>cardiffnlp/twitter-roberta-base-sentiment-latest</t>
-        </is>
-      </c>
-      <c r="D27" t="inlineStr">
-        <is>
-          <t>3-sentiment</t>
-        </is>
-      </c>
-      <c r="E27" t="n">
-        <v>46</v>
-      </c>
-      <c r="F27" t="n">
-        <v>50</v>
-      </c>
-      <c r="G27" t="n">
-        <v>0.92</v>
-      </c>
-      <c r="H27" t="n">
-        <v>1.2355</v>
-      </c>
-      <c r="I27" t="n">
-        <v>2.0197</v>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=-_-eIVAX1yQ</t>
-        </is>
-      </c>
-      <c r="B28" t="inlineStr">
-        <is>
-          <t>CardiffNLP Twitter RoBERTa</t>
-        </is>
-      </c>
-      <c r="C28" t="inlineStr">
-        <is>
-          <t>cardiffnlp/twitter-roberta-base-sentiment-latest</t>
-        </is>
-      </c>
-      <c r="D28" t="inlineStr">
-        <is>
-          <t>3-sentiment</t>
-        </is>
-      </c>
-      <c r="E28" t="n">
-        <v>29</v>
-      </c>
-      <c r="F28" t="n">
-        <v>50</v>
-      </c>
-      <c r="G28" t="n">
         <v>0.58</v>
-      </c>
-      <c r="H28" t="n">
-        <v>1.2355</v>
-      </c>
-      <c r="I28" t="n">
-        <v>2.0197</v>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=d2dgJGkw5p0</t>
-        </is>
-      </c>
-      <c r="B29" t="inlineStr">
-        <is>
-          <t>lxyuan DistilBERT Multilingual</t>
-        </is>
-      </c>
-      <c r="C29" t="inlineStr">
-        <is>
-          <t>lxyuan/distilbert-base-multilingual-cased-sentiments-student</t>
-        </is>
-      </c>
-      <c r="D29" t="inlineStr">
-        <is>
-          <t>3-sentiment</t>
-        </is>
-      </c>
-      <c r="E29" t="n">
-        <v>23</v>
-      </c>
-      <c r="F29" t="n">
-        <v>50</v>
-      </c>
-      <c r="G29" t="n">
-        <v>0.46</v>
-      </c>
-      <c r="H29" t="n">
-        <v>1.1556</v>
-      </c>
-      <c r="I29" t="n">
-        <v>0.8353</v>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=M8To7iorkxQ</t>
-        </is>
-      </c>
-      <c r="B30" t="inlineStr">
-        <is>
-          <t>lxyuan DistilBERT Multilingual</t>
-        </is>
-      </c>
-      <c r="C30" t="inlineStr">
-        <is>
-          <t>lxyuan/distilbert-base-multilingual-cased-sentiments-student</t>
-        </is>
-      </c>
-      <c r="D30" t="inlineStr">
-        <is>
-          <t>3-sentiment</t>
-        </is>
-      </c>
-      <c r="E30" t="n">
-        <v>37</v>
-      </c>
-      <c r="F30" t="n">
-        <v>50</v>
-      </c>
-      <c r="G30" t="n">
-        <v>0.74</v>
-      </c>
-      <c r="H30" t="n">
-        <v>1.1556</v>
-      </c>
-      <c r="I30" t="n">
-        <v>0.8353</v>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=-_-eIVAX1yQ</t>
-        </is>
-      </c>
-      <c r="B31" t="inlineStr">
-        <is>
-          <t>lxyuan DistilBERT Multilingual</t>
-        </is>
-      </c>
-      <c r="C31" t="inlineStr">
-        <is>
-          <t>lxyuan/distilbert-base-multilingual-cased-sentiments-student</t>
-        </is>
-      </c>
-      <c r="D31" t="inlineStr">
-        <is>
-          <t>3-sentiment</t>
-        </is>
-      </c>
-      <c r="E31" t="n">
-        <v>34</v>
-      </c>
-      <c r="F31" t="n">
-        <v>50</v>
-      </c>
-      <c r="G31" t="n">
-        <v>0.68</v>
-      </c>
-      <c r="H31" t="n">
-        <v>1.1556</v>
-      </c>
-      <c r="I31" t="n">
-        <v>0.8353</v>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=d2dgJGkw5p0</t>
-        </is>
-      </c>
-      <c r="B32" t="inlineStr">
-        <is>
-          <t>FiniteAutomata BERTweet</t>
-        </is>
-      </c>
-      <c r="C32" t="inlineStr">
-        <is>
-          <t>finiteautomata/bertweet-base-sentiment-analysis</t>
-        </is>
-      </c>
-      <c r="D32" t="inlineStr">
-        <is>
-          <t>3-sentiment</t>
-        </is>
-      </c>
-      <c r="E32" t="n">
-        <v>0</v>
-      </c>
-      <c r="F32" t="n">
-        <v>50</v>
-      </c>
-      <c r="G32" t="n">
-        <v>0</v>
-      </c>
-      <c r="H32" t="n">
-        <v>1.2548</v>
-      </c>
-      <c r="I32" t="n">
-        <v>1.7107</v>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=M8To7iorkxQ</t>
-        </is>
-      </c>
-      <c r="B33" t="inlineStr">
-        <is>
-          <t>FiniteAutomata BERTweet</t>
-        </is>
-      </c>
-      <c r="C33" t="inlineStr">
-        <is>
-          <t>finiteautomata/bertweet-base-sentiment-analysis</t>
-        </is>
-      </c>
-      <c r="D33" t="inlineStr">
-        <is>
-          <t>3-sentiment</t>
-        </is>
-      </c>
-      <c r="E33" t="n">
-        <v>0</v>
-      </c>
-      <c r="F33" t="n">
-        <v>50</v>
-      </c>
-      <c r="G33" t="n">
-        <v>0</v>
-      </c>
-      <c r="H33" t="n">
-        <v>1.2548</v>
-      </c>
-      <c r="I33" t="n">
-        <v>1.7107</v>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=-_-eIVAX1yQ</t>
-        </is>
-      </c>
-      <c r="B34" t="inlineStr">
-        <is>
-          <t>FiniteAutomata BERTweet</t>
-        </is>
-      </c>
-      <c r="C34" t="inlineStr">
-        <is>
-          <t>finiteautomata/bertweet-base-sentiment-analysis</t>
-        </is>
-      </c>
-      <c r="D34" t="inlineStr">
-        <is>
-          <t>3-sentiment</t>
-        </is>
-      </c>
-      <c r="E34" t="n">
-        <v>0</v>
-      </c>
-      <c r="F34" t="n">
-        <v>50</v>
-      </c>
-      <c r="G34" t="n">
-        <v>0</v>
-      </c>
-      <c r="H34" t="n">
-        <v>1.2548</v>
-      </c>
-      <c r="I34" t="n">
-        <v>1.7107</v>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" t="inlineStr">
-        <is>
-          <t>OVERALL</t>
-        </is>
-      </c>
-      <c r="B35" t="inlineStr">
-        <is>
-          <t>Pre-tuning baseline</t>
-        </is>
-      </c>
-      <c r="C35" t="inlineStr">
-        <is>
-          <t>j-hartmann/emotion-english-distilroberta-base</t>
-        </is>
-      </c>
-      <c r="D35" t="inlineStr">
-        <is>
-          <t>7-emotion</t>
-        </is>
-      </c>
-      <c r="E35" t="n">
-        <v>67</v>
-      </c>
-      <c r="F35" t="n">
-        <v>150</v>
-      </c>
-      <c r="G35" t="n">
-        <v>0.4467</v>
-      </c>
-      <c r="H35" t="n">
-        <v>1.2324</v>
-      </c>
-      <c r="I35" t="n">
-        <v>1.0282</v>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" t="inlineStr">
-        <is>
-          <t>OVERALL</t>
-        </is>
-      </c>
-      <c r="B36" t="inlineStr">
-        <is>
-          <t>GoEmotions fine-tuned</t>
-        </is>
-      </c>
-      <c r="C36" t="inlineStr">
-        <is>
-          <t>chase1zhang/youtube-emotion-distilbert</t>
-        </is>
-      </c>
-      <c r="D36" t="inlineStr">
-        <is>
-          <t>7-emotion</t>
-        </is>
-      </c>
-      <c r="E36" t="n">
-        <v>49</v>
-      </c>
-      <c r="F36" t="n">
-        <v>150</v>
-      </c>
-      <c r="G36" t="n">
-        <v>0.3267</v>
-      </c>
-      <c r="H36" t="n">
-        <v>0.0582</v>
-      </c>
-      <c r="I36" t="n">
-        <v>0.8488</v>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" t="inlineStr">
-        <is>
-          <t>OVERALL</t>
-        </is>
-      </c>
-      <c r="B37" t="inlineStr">
-        <is>
-          <t>YouTube-domain adapted (your model)</t>
-        </is>
-      </c>
-      <c r="C37" t="inlineStr">
-        <is>
-          <t>chase1zhang/youtube-emotion-distilbert-domain-adapted</t>
-        </is>
-      </c>
-      <c r="D37" t="inlineStr">
-        <is>
-          <t>7-emotion</t>
-        </is>
-      </c>
-      <c r="E37" t="n">
-        <v>84</v>
-      </c>
-      <c r="F37" t="n">
-        <v>150</v>
-      </c>
-      <c r="G37" t="n">
-        <v>0.5600000000000001</v>
-      </c>
-      <c r="H37" t="n">
-        <v>0.0385</v>
-      </c>
-      <c r="I37" t="n">
-        <v>0.9343</v>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" t="inlineStr">
-        <is>
-          <t>OVERALL</t>
-        </is>
-      </c>
-      <c r="B38" t="inlineStr">
-        <is>
-          <t>Public GoEmotions RoBERTa (SamLowe)</t>
-        </is>
-      </c>
-      <c r="C38" t="inlineStr">
-        <is>
-          <t>SamLowe/roberta-base-go_emotions</t>
-        </is>
-      </c>
-      <c r="D38" t="inlineStr">
-        <is>
-          <t>7-emotion</t>
-        </is>
-      </c>
-      <c r="E38" t="n">
-        <v>80</v>
-      </c>
-      <c r="F38" t="n">
-        <v>150</v>
-      </c>
-      <c r="G38" t="n">
-        <v>0.5333</v>
-      </c>
-      <c r="H38" t="n">
-        <v>0.9086</v>
-      </c>
-      <c r="I38" t="n">
-        <v>1.8941</v>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" t="inlineStr">
-        <is>
-          <t>OVERALL</t>
-        </is>
-      </c>
-      <c r="B39" t="inlineStr">
-        <is>
-          <t>Public RoBERTa-large 7-emotion</t>
-        </is>
-      </c>
-      <c r="C39" t="inlineStr">
-        <is>
-          <t>j-hartmann/emotion-english-roberta-large</t>
-        </is>
-      </c>
-      <c r="D39" t="inlineStr">
-        <is>
-          <t>7-emotion</t>
-        </is>
-      </c>
-      <c r="E39" t="n">
-        <v>62</v>
-      </c>
-      <c r="F39" t="n">
-        <v>150</v>
-      </c>
-      <c r="G39" t="n">
-        <v>0.4133</v>
-      </c>
-      <c r="H39" t="n">
-        <v>1.4107</v>
-      </c>
-      <c r="I39" t="n">
-        <v>7.1657</v>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" t="inlineStr">
-        <is>
-          <t>OVERALL</t>
-        </is>
-      </c>
-      <c r="B40" t="inlineStr">
-        <is>
-          <t>YouTube-domain adapted RoBERTa (SamLowe)</t>
-        </is>
-      </c>
-      <c r="C40" t="inlineStr">
-        <is>
-          <t>chase1zhang/youtube-emotion-samlowe-roberta-domain-adapted</t>
-        </is>
-      </c>
-      <c r="D40" t="inlineStr">
-        <is>
-          <t>7-emotion</t>
-        </is>
-      </c>
-      <c r="E40" t="n">
-        <v>93</v>
-      </c>
-      <c r="F40" t="n">
-        <v>150</v>
-      </c>
-      <c r="G40" t="n">
-        <v>0.62</v>
-      </c>
-      <c r="H40" t="n">
-        <v>0.1597</v>
-      </c>
-      <c r="I40" t="n">
-        <v>2.0179</v>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" t="inlineStr">
-        <is>
-          <t>OVERALL</t>
-        </is>
-      </c>
-      <c r="B41" t="inlineStr">
-        <is>
-          <t>YouTube-domain adapted DistilRoBERTa (j-hartmann)</t>
-        </is>
-      </c>
-      <c r="C41" t="inlineStr">
-        <is>
-          <t>chase1zhang/youtube-emotion-jhartmann-distilroberta-domain-adapted</t>
-        </is>
-      </c>
-      <c r="D41" t="inlineStr">
-        <is>
-          <t>7-emotion</t>
-        </is>
-      </c>
-      <c r="E41" t="n">
-        <v>83</v>
-      </c>
-      <c r="F41" t="n">
-        <v>150</v>
-      </c>
-      <c r="G41" t="n">
-        <v>0.5533</v>
-      </c>
-      <c r="H41" t="n">
-        <v>0.0912</v>
-      </c>
-      <c r="I41" t="n">
-        <v>1.0381</v>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" t="inlineStr">
-        <is>
-          <t>OVERALL</t>
-        </is>
-      </c>
-      <c r="B42" t="inlineStr">
-        <is>
-          <t>YouTube-domain adapted RoBERTa-large (j-hartmann)</t>
-        </is>
-      </c>
-      <c r="C42" t="inlineStr">
-        <is>
-          <t>chase1zhang/youtube-emotion-roberta-large-domain-adapted</t>
-        </is>
-      </c>
-      <c r="D42" t="inlineStr">
-        <is>
-          <t>7-emotion</t>
-        </is>
-      </c>
-      <c r="E42" t="n">
-        <v>94</v>
-      </c>
-      <c r="F42" t="n">
-        <v>150</v>
-      </c>
-      <c r="G42" t="n">
-        <v>0.6267</v>
-      </c>
-      <c r="H42" t="n">
-        <v>0.186</v>
-      </c>
-      <c r="I42" t="n">
-        <v>7.3825</v>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" t="inlineStr">
-        <is>
-          <t>OVERALL</t>
-        </is>
-      </c>
-      <c r="B43" t="inlineStr">
-        <is>
-          <t>CardiffNLP Twitter RoBERTa</t>
-        </is>
-      </c>
-      <c r="C43" t="inlineStr">
-        <is>
-          <t>cardiffnlp/twitter-roberta-base-sentiment-latest</t>
-        </is>
-      </c>
-      <c r="D43" t="inlineStr">
-        <is>
-          <t>3-sentiment</t>
-        </is>
-      </c>
-      <c r="E43" t="n">
-        <v>105</v>
-      </c>
-      <c r="F43" t="n">
-        <v>150</v>
-      </c>
-      <c r="G43" t="n">
-        <v>0.7</v>
-      </c>
-      <c r="H43" t="n">
-        <v>1.2355</v>
-      </c>
-      <c r="I43" t="n">
-        <v>2.0197</v>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" t="inlineStr">
-        <is>
-          <t>OVERALL</t>
-        </is>
-      </c>
-      <c r="B44" t="inlineStr">
-        <is>
-          <t>lxyuan DistilBERT Multilingual</t>
-        </is>
-      </c>
-      <c r="C44" t="inlineStr">
-        <is>
-          <t>lxyuan/distilbert-base-multilingual-cased-sentiments-student</t>
-        </is>
-      </c>
-      <c r="D44" t="inlineStr">
-        <is>
-          <t>3-sentiment</t>
-        </is>
-      </c>
-      <c r="E44" t="n">
-        <v>94</v>
-      </c>
-      <c r="F44" t="n">
-        <v>150</v>
-      </c>
-      <c r="G44" t="n">
-        <v>0.6267</v>
-      </c>
-      <c r="H44" t="n">
-        <v>1.1556</v>
-      </c>
-      <c r="I44" t="n">
-        <v>0.8353</v>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" t="inlineStr">
-        <is>
-          <t>OVERALL</t>
-        </is>
-      </c>
-      <c r="B45" t="inlineStr">
-        <is>
-          <t>FiniteAutomata BERTweet</t>
-        </is>
-      </c>
-      <c r="C45" t="inlineStr">
-        <is>
-          <t>finiteautomata/bertweet-base-sentiment-analysis</t>
-        </is>
-      </c>
-      <c r="D45" t="inlineStr">
-        <is>
-          <t>3-sentiment</t>
-        </is>
-      </c>
-      <c r="E45" t="n">
-        <v>0</v>
-      </c>
-      <c r="F45" t="n">
-        <v>150</v>
-      </c>
-      <c r="G45" t="n">
-        <v>0</v>
-      </c>
-      <c r="H45" t="n">
-        <v>1.2548</v>
-      </c>
-      <c r="I45" t="n">
-        <v>1.7107</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Fix remaining 150-comment references and clean up xlsx
- Remove Pipeline 3 from Experimental_results.xlsx (rule-based, not a tested model)
- Update Pipeline 2 sentiment section from 150-comment to 500-comment benchmark
- Fix conclusion sections: 105/150 → 334/500
- Fix Section 11.3 intro: 150-comment → 500-comment
- Update README: 150-comment → 500-comment benchmark

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/experiments/Experimental_results.xlsx
+++ b/experiments/Experimental_results.xlsx
@@ -423,11 +423,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A2:G79"/>
+  <dimension ref="A2:G71"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
-    <col width="43" customWidth="1" min="2" max="2"/>
+    <col width="45" customWidth="1" min="2" max="2"/>
     <col width="22" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
     <col width="22" customWidth="1" min="5" max="5"/>
@@ -614,7 +614,7 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>Trades in-domain accuracy for YouTube-domain performance</t>
+          <t>Trades in-domain for YouTube-domain</t>
         </is>
       </c>
     </row>
@@ -974,7 +974,7 @@
       </c>
       <c r="D36" s="1" t="inlineStr">
         <is>
-          <t>App benchmark (150)</t>
+          <t>App benchmark (500)</t>
         </is>
       </c>
       <c r="E36" s="1" t="inlineStr">
@@ -984,12 +984,7 @@
       </c>
       <c r="F36" s="1" t="inlineStr">
         <is>
-          <t>Runtime w/o loading</t>
-        </is>
-      </c>
-      <c r="G36" s="1" t="inlineStr">
-        <is>
-          <t>Purpose</t>
+          <t>Notes</t>
         </is>
       </c>
     </row>
@@ -1006,18 +1001,13 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>105/150</t>
+          <t>334/500</t>
         </is>
       </c>
       <c r="E37" t="n">
-        <v>0.7</v>
+        <v>0.668</v>
       </c>
       <c r="F37" t="inlineStr">
-        <is>
-          <t>1.9316s</t>
-        </is>
-      </c>
-      <c r="G37" t="inlineStr">
         <is>
           <t>Best accuracy; recommended</t>
         </is>
@@ -1036,18 +1026,13 @@
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>94/150</t>
+          <t>306/500</t>
         </is>
       </c>
       <c r="E38" t="n">
-        <v>0.6267</v>
+        <v>0.612</v>
       </c>
       <c r="F38" t="inlineStr">
-        <is>
-          <t>0.8794s</t>
-        </is>
-      </c>
-      <c r="G38" t="inlineStr">
         <is>
           <t>Fastest inference; multilingual</t>
         </is>
@@ -1066,655 +1051,532 @@
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>0/150*</t>
+          <t>228/500</t>
         </is>
       </c>
       <c r="E39" t="n">
-        <v>0</v>
+        <v>0.456</v>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>1.7399s</t>
-        </is>
-      </c>
-      <c r="G39" t="inlineStr">
-        <is>
-          <t>*Label format mismatch; output correct</t>
+          <t>Label format: POS/NEU/NEG; output correct</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="B42" t="inlineStr">
         <is>
-          <t>Pipeline 3 - Business Decision Engine (rule-based, combining emotion + sentiment)</t>
+          <t>Experiment 2: Assessing the overall app performance on Streamlit Cloud</t>
         </is>
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="1" t="n"/>
-      <c r="B43" s="1" t="inlineStr">
-        <is>
-          <t>Rule</t>
-        </is>
-      </c>
-      <c r="C43" s="1" t="inlineStr">
-        <is>
-          <t>Condition</t>
-        </is>
-      </c>
-      <c r="D43" s="1" t="inlineStr">
-        <is>
-          <t>Decision</t>
-        </is>
-      </c>
-      <c r="E43" s="1" t="inlineStr">
-        <is>
-          <t>Risk Level</t>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>App URL</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>https://youtube-emotion-analyzer.streamlit.app/</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="B44" t="inlineStr">
         <is>
-          <t>High Risk</t>
+          <t>Benchmark</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Negative emotion ratio &gt;= 40% OR Negative sentiment ratio &gt;= 40%</t>
-        </is>
-      </c>
-      <c r="D44" t="inlineStr">
-        <is>
-          <t>Review before scaling</t>
-        </is>
-      </c>
-      <c r="E44" t="inlineStr">
-        <is>
-          <t>High</t>
+          <t>500 comments across 10 YouTube videos (150 manually reviewed + 350 DeepSeek-labeled)</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="B45" t="inlineStr">
         <is>
-          <t>Low Risk</t>
+          <t>Benchmark file</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Dominant emotion is Joy/Surprise AND Positive sentiment ratio &gt;= 50%</t>
-        </is>
-      </c>
-      <c r="D45" t="inlineStr">
-        <is>
-          <t>Scale positive creative</t>
-        </is>
-      </c>
-      <c r="E45" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-    </row>
-    <row r="46">
-      <c r="B46" t="inlineStr">
-        <is>
-          <t>Medium Risk (engagement)</t>
-        </is>
-      </c>
-      <c r="C46" t="inlineStr">
-        <is>
-          <t>Dominant emotion is Neutral</t>
-        </is>
-      </c>
-      <c r="D46" t="inlineStr">
-        <is>
-          <t>Improve engagement hook</t>
-        </is>
-      </c>
-      <c r="E46" t="inlineStr">
-        <is>
-          <t>Medium</t>
+          <t>data/app_per_comment_manual_labels_500.csv</t>
         </is>
       </c>
     </row>
     <row r="47">
-      <c r="B47" t="inlineStr">
-        <is>
-          <t>Medium Risk (mixed)</t>
-        </is>
-      </c>
-      <c r="C47" t="inlineStr">
-        <is>
-          <t>All other mixed signals</t>
-        </is>
-      </c>
-      <c r="D47" t="inlineStr">
-        <is>
-          <t>Monitor and review samples</t>
-        </is>
-      </c>
-      <c r="E47" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
+      <c r="A47" s="1" t="n"/>
+      <c r="B47" s="1" t="inlineStr">
+        <is>
+          <t>Task</t>
+        </is>
+      </c>
+      <c r="C47" s="1" t="inlineStr">
+        <is>
+          <t>Model / Pipeline</t>
+        </is>
+      </c>
+      <c r="D47" s="1" t="inlineStr">
+        <is>
+          <t>Matched / 500</t>
+        </is>
+      </c>
+      <c r="E47" s="1" t="inlineStr">
+        <is>
+          <t>Accuracy</t>
+        </is>
+      </c>
+      <c r="F47" s="1" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>7-emotion</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>Pre-tuning baseline</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>179/500</t>
+        </is>
+      </c>
+      <c r="E48" t="n">
+        <v>0.358</v>
+      </c>
+      <c r="F48" t="inlineStr"/>
+    </row>
+    <row r="49">
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>7-emotion</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>GoEmotions fine-tuned</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>141/500</t>
+        </is>
+      </c>
+      <c r="E49" t="n">
+        <v>0.282</v>
+      </c>
+      <c r="F49" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="B50" t="inlineStr">
         <is>
-          <t>Experiment 2: Assessing the overall app performance on Streamlit Cloud</t>
+          <t>7-emotion</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>YouTube-domain adapted DistilBERT</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>317/500</t>
+        </is>
+      </c>
+      <c r="E50" t="n">
+        <v>0.634</v>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>Best project-owned 7-emotion</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="B51" t="inlineStr">
         <is>
-          <t>App URL</t>
+          <t>7-emotion</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>https://youtube-emotion-analyzer.streamlit.app/</t>
-        </is>
-      </c>
+          <t>Public GoEmotions RoBERTa</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>208/500</t>
+        </is>
+      </c>
+      <c r="E51" t="n">
+        <v>0.416</v>
+      </c>
+      <c r="F51" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="B52" t="inlineStr">
         <is>
-          <t>Benchmark</t>
+          <t>7-emotion</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>500 comments across 10 YouTube videos (150 manually reviewed + 350 DeepSeek-labeled)</t>
-        </is>
-      </c>
+          <t>Public RoBERTa-large</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>185/500</t>
+        </is>
+      </c>
+      <c r="E52" t="n">
+        <v>0.37</v>
+      </c>
+      <c r="F52" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="B53" t="inlineStr">
         <is>
-          <t>Benchmark file</t>
+          <t>7-emotion</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>data/app_per_comment_manual_labels_500.csv</t>
-        </is>
-      </c>
+          <t>YouTube-domain adapted RoBERTa</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>315/500</t>
+        </is>
+      </c>
+      <c r="E53" t="n">
+        <v>0.63</v>
+      </c>
+      <c r="F53" t="inlineStr"/>
+    </row>
+    <row r="54">
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>7-emotion</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>YouTube-domain adapted DistilRoBERTa</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>306/500</t>
+        </is>
+      </c>
+      <c r="E54" t="n">
+        <v>0.612</v>
+      </c>
+      <c r="F54" t="inlineStr"/>
     </row>
     <row r="55">
-      <c r="A55" s="1" t="n"/>
-      <c r="B55" s="1" t="inlineStr">
-        <is>
-          <t>Task</t>
-        </is>
-      </c>
-      <c r="C55" s="1" t="inlineStr">
-        <is>
-          <t>Model / Pipeline</t>
-        </is>
-      </c>
-      <c r="D55" s="1" t="inlineStr">
-        <is>
-          <t>Matched / 500</t>
-        </is>
-      </c>
-      <c r="E55" s="1" t="inlineStr">
-        <is>
-          <t>Accuracy</t>
-        </is>
-      </c>
-      <c r="F55" s="1" t="inlineStr">
-        <is>
-          <t>Notes</t>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>3-sentiment</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>CardiffNLP sentiment pipeline</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>334/500</t>
+        </is>
+      </c>
+      <c r="E55" t="n">
+        <v>0.668</v>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>Best overall signal</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="B56" t="inlineStr">
         <is>
-          <t>7-emotion</t>
+          <t>3-sentiment</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>Pre-tuning baseline</t>
+          <t>lxyuan sentiment</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>179/500</t>
+          <t>306/500</t>
         </is>
       </c>
       <c r="E56" t="n">
-        <v>0.358</v>
+        <v>0.612</v>
       </c>
       <c r="F56" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="B57" t="inlineStr">
         <is>
-          <t>7-emotion</t>
+          <t>3-sentiment</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>GoEmotions fine-tuned</t>
+          <t>BERTweet sentiment</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>141/500</t>
+          <t>228/500</t>
         </is>
       </c>
       <c r="E57" t="n">
-        <v>0.282</v>
+        <v>0.456</v>
       </c>
       <c r="F57" t="inlineStr"/>
-    </row>
-    <row r="58">
-      <c r="B58" t="inlineStr">
-        <is>
-          <t>7-emotion</t>
-        </is>
-      </c>
-      <c r="C58" t="inlineStr">
-        <is>
-          <t>YouTube-domain adapted DistilBERT</t>
-        </is>
-      </c>
-      <c r="D58" t="inlineStr">
-        <is>
-          <t>317/500</t>
-        </is>
-      </c>
-      <c r="E58" t="n">
-        <v>0.634</v>
-      </c>
-      <c r="F58" t="inlineStr">
-        <is>
-          <t>Best project-owned 7-emotion</t>
-        </is>
-      </c>
-    </row>
-    <row r="59">
-      <c r="B59" t="inlineStr">
-        <is>
-          <t>7-emotion</t>
-        </is>
-      </c>
-      <c r="C59" t="inlineStr">
-        <is>
-          <t>Public GoEmotions RoBERTa</t>
-        </is>
-      </c>
-      <c r="D59" t="inlineStr">
-        <is>
-          <t>208/500</t>
-        </is>
-      </c>
-      <c r="E59" t="n">
-        <v>0.416</v>
-      </c>
-      <c r="F59" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="B60" t="inlineStr">
         <is>
-          <t>7-emotion</t>
-        </is>
-      </c>
-      <c r="C60" t="inlineStr">
-        <is>
-          <t>Public RoBERTa-large</t>
-        </is>
-      </c>
-      <c r="D60" t="inlineStr">
-        <is>
-          <t>185/500</t>
-        </is>
-      </c>
-      <c r="E60" t="n">
-        <v>0.37</v>
-      </c>
-      <c r="F60" t="inlineStr"/>
+          <t>Per-video accuracy: YouTube-domain adapted DistilBERT (best project-owned model)</t>
+        </is>
+      </c>
     </row>
     <row r="61">
-      <c r="B61" t="inlineStr">
-        <is>
-          <t>7-emotion</t>
-        </is>
-      </c>
-      <c r="C61" t="inlineStr">
-        <is>
-          <t>YouTube-domain adapted RoBERTa</t>
-        </is>
-      </c>
-      <c r="D61" t="inlineStr">
-        <is>
-          <t>315/500</t>
-        </is>
-      </c>
-      <c r="E61" t="n">
-        <v>0.63</v>
-      </c>
-      <c r="F61" t="inlineStr"/>
+      <c r="A61" s="1" t="n"/>
+      <c r="B61" s="1" t="inlineStr">
+        <is>
+          <t>Video</t>
+        </is>
+      </c>
+      <c r="C61" s="1" t="inlineStr">
+        <is>
+          <t>Matched / 50</t>
+        </is>
+      </c>
+      <c r="D61" s="1" t="inlineStr">
+        <is>
+          <t>Accuracy</t>
+        </is>
+      </c>
+      <c r="E61" s="1" t="inlineStr">
+        <is>
+          <t>Manual main label</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="B62" t="inlineStr">
         <is>
-          <t>7-emotion</t>
+          <t>rare_earths</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>YouTube-domain adapted DistilRoBERTa</t>
-        </is>
-      </c>
-      <c r="D62" t="inlineStr">
-        <is>
-          <t>306/500</t>
-        </is>
-      </c>
-      <c r="E62" t="n">
-        <v>0.612</v>
-      </c>
-      <c r="F62" t="inlineStr"/>
+          <t>28/50</t>
+        </is>
+      </c>
+      <c r="D62" t="n">
+        <v>0.5600000000000001</v>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="B63" t="inlineStr">
         <is>
-          <t>3-sentiment</t>
+          <t>avatar_clip</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>CardiffNLP sentiment pipeline</t>
-        </is>
-      </c>
-      <c r="D63" t="inlineStr">
-        <is>
-          <t>334/500</t>
-        </is>
-      </c>
-      <c r="E63" t="n">
-        <v>0.668</v>
-      </c>
-      <c r="F63" t="inlineStr">
-        <is>
-          <t>Best overall signal</t>
+          <t>37/50</t>
+        </is>
+      </c>
+      <c r="D63" t="n">
+        <v>0.74</v>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>joy</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="B64" t="inlineStr">
         <is>
-          <t>3-sentiment</t>
+          <t>shooting_news</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>lxyuan sentiment</t>
-        </is>
-      </c>
-      <c r="D64" t="inlineStr">
-        <is>
-          <t>306/500</t>
-        </is>
-      </c>
-      <c r="E64" t="n">
-        <v>0.612</v>
-      </c>
-      <c r="F64" t="inlineStr"/>
+          <t>17/50</t>
+        </is>
+      </c>
+      <c r="D64" t="n">
+        <v>0.34</v>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>anger</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="B65" t="inlineStr">
         <is>
-          <t>3-sentiment</t>
+          <t>anger_brand_crisis</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>BERTweet sentiment</t>
-        </is>
-      </c>
-      <c r="D65" t="inlineStr">
-        <is>
-          <t>228/500</t>
-        </is>
-      </c>
-      <c r="E65" t="n">
-        <v>0.456</v>
-      </c>
-      <c r="F65" t="inlineStr"/>
+          <t>36/50</t>
+        </is>
+      </c>
+      <c r="D65" t="n">
+        <v>0.72</v>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>anger</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>fear_public_safety</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>25/50</t>
+        </is>
+      </c>
+      <c r="D66" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>fear</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>sadness_psa</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>37/50</t>
+        </is>
+      </c>
+      <c r="D67" t="n">
+        <v>0.74</v>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>sadness</t>
+        </is>
+      </c>
     </row>
     <row r="68">
       <c r="B68" t="inlineStr">
         <is>
-          <t>Per-video accuracy: YouTube-domain adapted DistilBERT (best project-owned model)</t>
+          <t>surprise_product_fail</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>36/50</t>
+        </is>
+      </c>
+      <c r="D68" t="n">
+        <v>0.72</v>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>surprise</t>
         </is>
       </c>
     </row>
     <row r="69">
-      <c r="A69" s="1" t="n"/>
-      <c r="B69" s="1" t="inlineStr">
-        <is>
-          <t>Video</t>
-        </is>
-      </c>
-      <c r="C69" s="1" t="inlineStr">
-        <is>
-          <t>Matched / 50</t>
-        </is>
-      </c>
-      <c r="D69" s="1" t="inlineStr">
-        <is>
-          <t>Accuracy</t>
-        </is>
-      </c>
-      <c r="E69" s="1" t="inlineStr">
-        <is>
-          <t>Manual main label</t>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>disgust_food_safety</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>36/50</t>
+        </is>
+      </c>
+      <c r="D69" t="n">
+        <v>0.72</v>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>disgust</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="B70" t="inlineStr">
         <is>
-          <t>rare_earths</t>
+          <t>joy_trailer</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>28/50</t>
+          <t>33/50</t>
         </is>
       </c>
       <c r="D70" t="n">
-        <v>0.5600000000000001</v>
+        <v>0.66</v>
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>neutral</t>
+          <t>joy</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="B71" t="inlineStr">
         <is>
-          <t>avatar_clip</t>
+          <t>brand_crisis_negative</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>37/50</t>
+          <t>32/50</t>
         </is>
       </c>
       <c r="D71" t="n">
-        <v>0.74</v>
+        <v>0.64</v>
       </c>
       <c r="E71" t="inlineStr">
-        <is>
-          <t>joy</t>
-        </is>
-      </c>
-    </row>
-    <row r="72">
-      <c r="B72" t="inlineStr">
-        <is>
-          <t>shooting_news</t>
-        </is>
-      </c>
-      <c r="C72" t="inlineStr">
-        <is>
-          <t>17/50</t>
-        </is>
-      </c>
-      <c r="D72" t="n">
-        <v>0.34</v>
-      </c>
-      <c r="E72" t="inlineStr">
-        <is>
-          <t>anger</t>
-        </is>
-      </c>
-    </row>
-    <row r="73">
-      <c r="B73" t="inlineStr">
-        <is>
-          <t>anger_brand_crisis</t>
-        </is>
-      </c>
-      <c r="C73" t="inlineStr">
-        <is>
-          <t>36/50</t>
-        </is>
-      </c>
-      <c r="D73" t="n">
-        <v>0.72</v>
-      </c>
-      <c r="E73" t="inlineStr">
-        <is>
-          <t>anger</t>
-        </is>
-      </c>
-    </row>
-    <row r="74">
-      <c r="B74" t="inlineStr">
-        <is>
-          <t>fear_public_safety</t>
-        </is>
-      </c>
-      <c r="C74" t="inlineStr">
-        <is>
-          <t>25/50</t>
-        </is>
-      </c>
-      <c r="D74" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="E74" t="inlineStr">
-        <is>
-          <t>fear</t>
-        </is>
-      </c>
-    </row>
-    <row r="75">
-      <c r="B75" t="inlineStr">
-        <is>
-          <t>sadness_psa</t>
-        </is>
-      </c>
-      <c r="C75" t="inlineStr">
-        <is>
-          <t>37/50</t>
-        </is>
-      </c>
-      <c r="D75" t="n">
-        <v>0.74</v>
-      </c>
-      <c r="E75" t="inlineStr">
-        <is>
-          <t>sadness</t>
-        </is>
-      </c>
-    </row>
-    <row r="76">
-      <c r="B76" t="inlineStr">
-        <is>
-          <t>surprise_product_fail</t>
-        </is>
-      </c>
-      <c r="C76" t="inlineStr">
-        <is>
-          <t>36/50</t>
-        </is>
-      </c>
-      <c r="D76" t="n">
-        <v>0.72</v>
-      </c>
-      <c r="E76" t="inlineStr">
-        <is>
-          <t>surprise</t>
-        </is>
-      </c>
-    </row>
-    <row r="77">
-      <c r="B77" t="inlineStr">
-        <is>
-          <t>disgust_food_safety</t>
-        </is>
-      </c>
-      <c r="C77" t="inlineStr">
-        <is>
-          <t>36/50</t>
-        </is>
-      </c>
-      <c r="D77" t="n">
-        <v>0.72</v>
-      </c>
-      <c r="E77" t="inlineStr">
-        <is>
-          <t>disgust</t>
-        </is>
-      </c>
-    </row>
-    <row r="78">
-      <c r="B78" t="inlineStr">
-        <is>
-          <t>joy_trailer</t>
-        </is>
-      </c>
-      <c r="C78" t="inlineStr">
-        <is>
-          <t>33/50</t>
-        </is>
-      </c>
-      <c r="D78" t="n">
-        <v>0.66</v>
-      </c>
-      <c r="E78" t="inlineStr">
-        <is>
-          <t>joy</t>
-        </is>
-      </c>
-    </row>
-    <row r="79">
-      <c r="B79" t="inlineStr">
-        <is>
-          <t>brand_crisis_negative</t>
-        </is>
-      </c>
-      <c r="C79" t="inlineStr">
-        <is>
-          <t>32/50</t>
-        </is>
-      </c>
-      <c r="D79" t="n">
-        <v>0.64</v>
-      </c>
-      <c r="E79" t="inlineStr">
         <is>
           <t>anger</t>
         </is>

</xml_diff>